<commit_message>
Correção de algumas partes de código
</commit_message>
<xml_diff>
--- a/tabela_completa_com_cotacao.xlsx
+++ b/tabela_completa_com_cotacao.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,7 +509,7 @@
         <v>1234</v>
       </c>
       <c r="I2" t="n">
-        <v>5.14</v>
+        <v>5.16</v>
       </c>
       <c r="J2" t="n">
         <v>5555</v>
@@ -569,50 +569,101 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FTR-003</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>600</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>SEM VALOR</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>SEM VALOR</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>159.35</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>SEM VALOR</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>SEM VALOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Proprietario_teste</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>FTR-001</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>FTR-004</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>GBP</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E5" t="n">
         <v>9343.9</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>PENDENTE</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>SEM VALOR</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>SEM VALOR</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>SEM VALOR</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>SEM VALOR</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>SEM VALOR</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>SEM VALOR</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>SEM VALOR</t>
         </is>

</xml_diff>